<commit_message>
fix(samples): let the second coverage-3 version accept submission code D
Version 1 and version 2 both limited the submission code to A, B or C,
so submission D could not be entered. Version 2 now accepts D, and its
version number moves to 2610120003 so it can replace an upload of the
earlier file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/coverage3/ctosim_coverage3_v2.xlsx
+++ b/samples/coverage3/ctosim_coverage3_v2.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -725,17 +725,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Submission code: type A, B or C as told in the instructions</t>
+          <t>Submission code: type D (version 2)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>regex(., '^[ABC]$')</t>
+          <t>regex(., '^[ABCD]$')</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>A, B or C</t>
+          <t>A, B, C or D</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2610120002</t>
+          <t>2610120003</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>